<commit_message>
v1.2.9 pt3 completo + btn atrás
</commit_message>
<xml_diff>
--- a/output/EIRL ADVANCED LOGISTICS GROUP (ALG).xlsx
+++ b/output/EIRL ADVANCED LOGISTICS GROUP (ALG).xlsx
@@ -1527,7 +1527,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-43470627</t>
+          <t>2026-43464373</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-43456475</t>
+          <t>2026-43470627</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-43464373</t>
+          <t>2026-43456475</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-42860973</t>
+          <t>2026-42862348</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-42862348</t>
+          <t>2026-42860973</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-48585700</t>
+          <t>2026-48588019</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-48588019</t>
+          <t>2026-48585700</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">

</xml_diff>